<commit_message>
cleaning the data in excel
</commit_message>
<xml_diff>
--- a/raw_data/Data Cleaning Start.xlsx
+++ b/raw_data/Data Cleaning Start.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10514"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kenjifarre/Desktop/Create/1. Video/1. YouTube/1. Videos/122. Data Cleaning/2. Footage/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9fc9985745544391/Desktop/Data Engineering/Excel Data_cleaning/Excel_data_cleaning/raw_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7DC79FA-DFE3-E94D-857C-94159278F052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{C7DC79FA-DFE3-E94D-857C-94159278F052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BE39C8F-24A6-4D11-A549-B0575FA27CEB}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="21900" xr2:uid="{7F7E1DDE-3781-814A-825E-072C922D74F6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{7F7E1DDE-3781-814A-825E-072C922D74F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover Page" sheetId="3" r:id="rId1"/>
     <sheet name="Sheet1 (2)" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1 (3)" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,8 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="143">
   <si>
     <t>Date</t>
   </si>
@@ -310,16 +309,208 @@
   <si>
     <t>Made by Career Principles Ltd.</t>
   </si>
+  <si>
+    <t>client</t>
+  </si>
+  <si>
+    <t xml:space="preserve">amazon.com, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">tesla, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">netflix, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">the procter &amp; gamble company </t>
+  </si>
+  <si>
+    <t xml:space="preserve">the goldman sachs group, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">jpmorgan chase &amp; co. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">morgan stanley </t>
+  </si>
+  <si>
+    <t xml:space="preserve">citigroup inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">bank of america corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">walmart inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">target corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">costco wholesale corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">mcdonald's corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">exxon mobil corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">verizon communications inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">the home depot, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">cisco systems, inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">chevron corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">at&amp;t inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">intel corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">general motors company </t>
+  </si>
+  <si>
+    <t xml:space="preserve">microsoft corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">comcast corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">dell technologies inc. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">johnson &amp; johnson </t>
+  </si>
+  <si>
+    <t xml:space="preserve">fedex corporation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">general electric company </t>
+  </si>
+  <si>
+    <t xml:space="preserve">lockheed martin corporation </t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>contact</t>
+  </si>
+  <si>
+    <t>Bill Smith</t>
+  </si>
+  <si>
+    <t>Ken Singh</t>
+  </si>
+  <si>
+    <t>Harley Fritz</t>
+  </si>
+  <si>
+    <t>David Rasmussen</t>
+  </si>
+  <si>
+    <t>Ivan Hiney</t>
+  </si>
+  <si>
+    <t>Jonha Ma</t>
+  </si>
+  <si>
+    <t>Jordan Boone</t>
+  </si>
+  <si>
+    <t>Brendan Wallace</t>
+  </si>
+  <si>
+    <t>Conor Wise</t>
+  </si>
+  <si>
+    <t>Steven Michael</t>
+  </si>
+  <si>
+    <t>Jose Roach</t>
+  </si>
+  <si>
+    <t>Franklin Wrigt</t>
+  </si>
+  <si>
+    <t>Alia Thornton</t>
+  </si>
+  <si>
+    <t>Denzel Flores</t>
+  </si>
+  <si>
+    <t>Bruno Cordova</t>
+  </si>
+  <si>
+    <t>Jaylynn Napp</t>
+  </si>
+  <si>
+    <t>Bruce Rich</t>
+  </si>
+  <si>
+    <t>Arturo Moore</t>
+  </si>
+  <si>
+    <t>Bryce Carpenter</t>
+  </si>
+  <si>
+    <t>Jaidyn Andersen</t>
+  </si>
+  <si>
+    <t>Mark Walm</t>
+  </si>
+  <si>
+    <t>Harry Lee</t>
+  </si>
+  <si>
+    <t>Josh Johnson</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Cloud Tech</t>
+  </si>
+  <si>
+    <t>Texas</t>
+  </si>
+  <si>
+    <t>Strategy</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>Operations</t>
+  </si>
+  <si>
+    <t>Florida</t>
+  </si>
+  <si>
+    <t>Big Data</t>
+  </si>
+  <si>
+    <t>California</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -396,8 +587,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -413,6 +611,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -526,12 +730,12 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -574,11 +778,15 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Per cent" xfId="1" builtinId="5"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -941,95 +1149,95 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F288F16A-B5AF-2A4A-A64E-4CF0DB39CED4}">
   <dimension ref="B3:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="8"/>
+    <col min="1" max="1" width="10.875" style="8"/>
     <col min="2" max="2" width="8.5" style="8" customWidth="1"/>
-    <col min="3" max="3" width="102.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="102.625" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.5" style="8" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="8"/>
+    <col min="5" max="16384" width="10.875" style="8"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:4" ht="92" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:4" ht="92.25" x14ac:dyDescent="0.25">
       <c r="B3" s="5"/>
       <c r="C3" s="6" t="s">
         <v>76</v>
       </c>
       <c r="D3" s="7"/>
     </row>
-    <row r="4" spans="2:4" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:4" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="9"/>
       <c r="C4" s="10"/>
       <c r="D4" s="11"/>
     </row>
-    <row r="5" spans="2:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="9"/>
       <c r="C5" s="10"/>
       <c r="D5" s="11"/>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="9"/>
       <c r="C6"/>
       <c r="D6" s="11"/>
     </row>
-    <row r="7" spans="2:4" s="14" customFormat="1" ht="21" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" s="14" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="B7" s="12"/>
       <c r="C7" s="25" t="s">
         <v>72</v>
       </c>
       <c r="D7" s="13"/>
     </row>
-    <row r="8" spans="2:4" s="14" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
       <c r="C8" s="15"/>
       <c r="D8" s="13"/>
     </row>
-    <row r="9" spans="2:4" s="18" customFormat="1" ht="26" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:4" s="18" customFormat="1" ht="26.25" x14ac:dyDescent="0.25">
       <c r="B9" s="16"/>
       <c r="C9" s="26" t="s">
         <v>73</v>
       </c>
       <c r="D9" s="17"/>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="9"/>
       <c r="C10"/>
       <c r="D10" s="11"/>
     </row>
-    <row r="11" spans="2:4" ht="19" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B11" s="9"/>
       <c r="C11" s="19" t="s">
         <v>78</v>
       </c>
       <c r="D11" s="11"/>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="9"/>
       <c r="C12"/>
       <c r="D12" s="11"/>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="9"/>
       <c r="C13" s="20" t="s">
         <v>74</v>
       </c>
       <c r="D13" s="11"/>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="9"/>
       <c r="C14" t="s">
         <v>77</v>
       </c>
       <c r="D14" s="11"/>
     </row>
-    <row r="15" spans="2:4" ht="34" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:4" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B15" s="9"/>
       <c r="C15" s="21" t="s">
         <v>75</v>
       </c>
       <c r="D15" s="11"/>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="22"/>
       <c r="C16" s="23"/>
       <c r="D16" s="24"/>
@@ -1048,17 +1256,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD37A31F-92F2-FA4A-B7ED-0F04A433817B}">
   <dimension ref="B2:I42"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" customWidth="1"/>
-    <col min="2" max="2" width="7.1640625" customWidth="1"/>
+    <col min="1" max="1" width="6.625" customWidth="1"/>
+    <col min="2" max="2" width="7.125" customWidth="1"/>
     <col min="3" max="3" width="11" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="6.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.625" customWidth="1"/>
     <col min="9" max="9" width="5.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -1084,7 +1292,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="4">
         <v>45076</v>
       </c>
@@ -1111,7 +1319,7 @@
         <v>0.13288888888888889</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="4">
         <v>45076</v>
       </c>
@@ -1138,7 +1346,7 @@
         <v>0.27500000000000002</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="4">
         <v>45076</v>
       </c>
@@ -1162,7 +1370,7 @@
         <v>0.2717845117845118</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="4">
         <v>45076</v>
       </c>
@@ -1184,7 +1392,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="4">
         <v>45076</v>
       </c>
@@ -1211,7 +1419,7 @@
         <v>0.1368</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:9" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="4">
         <v>45077</v>
       </c>
@@ -1238,7 +1446,7 @@
         <v>8.9180327868852466E-2</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B9" s="4">
         <v>45077</v>
       </c>
@@ -1265,7 +1473,7 @@
         <v>0.14486486486486486</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B10" s="4">
         <v>45077</v>
       </c>
@@ -1292,7 +1500,7 @@
         <v>0.53815789473684206</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="4">
         <v>45077</v>
       </c>
@@ -1319,7 +1527,7 @@
         <v>0.43444444444444447</v>
       </c>
     </row>
-    <row r="12" spans="2:9" ht="44" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:9" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="4">
         <v>45077</v>
       </c>
@@ -1346,7 +1554,7 @@
         <v>0.23921568627450981</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="4">
         <v>45077</v>
       </c>
@@ -1373,7 +1581,7 @@
         <v>0.30210526315789471</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="4">
         <v>45077</v>
       </c>
@@ -1400,7 +1608,7 @@
         <v>0.16633333333333333</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" s="4">
         <v>45077</v>
       </c>
@@ -1427,7 +1635,7 @@
         <v>0.17333333333333334</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="4">
         <v>45078</v>
       </c>
@@ -1452,7 +1660,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="4">
         <v>45078</v>
       </c>
@@ -1479,7 +1687,7 @@
         <v>0.32915824915824915</v>
       </c>
     </row>
-    <row r="18" spans="2:9" ht="38" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:9" ht="38.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="4">
         <v>45078</v>
       </c>
@@ -1506,7 +1714,7 @@
         <v>0.21515151515151515</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="4">
         <v>45078</v>
       </c>
@@ -1533,7 +1741,7 @@
         <v>0.17052631578947369</v>
       </c>
     </row>
-    <row r="20" spans="2:9" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="4">
         <v>45078</v>
       </c>
@@ -1560,7 +1768,7 @@
         <v>0.12745901639344262</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="4">
         <v>45077</v>
       </c>
@@ -1587,7 +1795,7 @@
         <v>0.16633333333333333</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" s="4">
         <v>45077</v>
       </c>
@@ -1614,7 +1822,7 @@
         <v>0.17333333333333334</v>
       </c>
     </row>
-    <row r="23" spans="2:9" ht="8" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:9" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="4">
         <v>45078</v>
       </c>
@@ -1641,7 +1849,7 @@
         <v>0.12874692874692875</v>
       </c>
     </row>
-    <row r="24" spans="2:9" ht="96" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:9" ht="96" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="4">
         <v>45078</v>
       </c>
@@ -1668,7 +1876,7 @@
         <v>0.16044444444444445</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" s="4">
         <v>45078</v>
       </c>
@@ -1695,7 +1903,7 @@
         <v>0.21199999999999999</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="4">
         <v>45079</v>
       </c>
@@ -1722,7 +1930,7 @@
         <v>0.25695238095238093</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" s="4">
         <v>45079</v>
       </c>
@@ -1749,7 +1957,7 @@
         <v>0.19815384615384615</v>
       </c>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" s="4">
         <v>45079</v>
       </c>
@@ -1776,7 +1984,7 @@
         <v>0.22186666666666666</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" s="4">
         <v>45079</v>
       </c>
@@ -1803,7 +2011,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" s="4">
         <v>45079</v>
       </c>
@@ -1830,7 +2038,7 @@
         <v>0.21643243243243243</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" s="4">
         <v>45079</v>
       </c>
@@ -1857,7 +2065,7 @@
         <v>0.21333333333333335</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" s="4">
         <v>45079</v>
       </c>
@@ -1884,7 +2092,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" s="4">
         <v>45076</v>
       </c>
@@ -1911,32 +2119,1094 @@
         <v>0.1368</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="G34" s="1"/>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="G35" s="1"/>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="G36" s="1"/>
     </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="G37" s="1"/>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="G38" s="1"/>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="G39" s="1"/>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
       <c r="G40" s="1"/>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
       <c r="G41" s="1"/>
     </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
       <c r="G42" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC5C7CD2-DDEE-49A3-8DBD-614DFB6DF2AC}">
+  <dimension ref="B2:J42"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.625" customWidth="1"/>
+    <col min="2" max="2" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.75" customWidth="1"/>
+    <col min="4" max="4" width="19.375" customWidth="1"/>
+    <col min="5" max="5" width="19.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.375" customWidth="1"/>
+    <col min="7" max="7" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B2" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="E2" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="28" t="s">
+        <v>133</v>
+      </c>
+      <c r="G2" s="28" t="s">
+        <v>47</v>
+      </c>
+      <c r="H2" s="28" t="s">
+        <v>2</v>
+      </c>
+      <c r="I2" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B3" s="4">
+        <v>45076</v>
+      </c>
+      <c r="C3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F3" t="s">
+        <v>135</v>
+      </c>
+      <c r="G3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H3" s="1">
+        <v>4500</v>
+      </c>
+      <c r="I3" s="1">
+        <v>598</v>
+      </c>
+      <c r="J3" s="2">
+        <f>IFERROR(I3/H3,"N/A")</f>
+        <v>0.13288888888888889</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B4" s="4">
+        <v>45076</v>
+      </c>
+      <c r="C4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" t="s">
+        <v>111</v>
+      </c>
+      <c r="E4" t="s">
+        <v>136</v>
+      </c>
+      <c r="F4" t="s">
+        <v>137</v>
+      </c>
+      <c r="G4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H4" s="1">
+        <v>3800</v>
+      </c>
+      <c r="I4" s="1">
+        <v>1045</v>
+      </c>
+      <c r="J4" s="2">
+        <f t="shared" ref="J4:J35" si="0">IFERROR(I4/H4,"N/A")</f>
+        <v>0.27500000000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B5" s="4">
+        <v>45076</v>
+      </c>
+      <c r="C5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F5" t="s">
+        <v>137</v>
+      </c>
+      <c r="G5" t="s">
+        <v>142</v>
+      </c>
+      <c r="H5" s="1">
+        <v>3712.5</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1009</v>
+      </c>
+      <c r="J5" s="2">
+        <f t="shared" si="0"/>
+        <v>0.2717845117845118</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B6" s="4">
+        <v>45076</v>
+      </c>
+      <c r="C6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" t="s">
+        <v>138</v>
+      </c>
+      <c r="F6" t="s">
+        <v>139</v>
+      </c>
+      <c r="G6" t="s">
+        <v>142</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I6" s="1">
+        <v>779</v>
+      </c>
+      <c r="J6" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B7" s="4">
+        <v>45076</v>
+      </c>
+      <c r="C7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E7" t="s">
+        <v>138</v>
+      </c>
+      <c r="F7" t="s">
+        <v>139</v>
+      </c>
+      <c r="G7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="1">
+        <v>5000</v>
+      </c>
+      <c r="I7" s="1">
+        <v>684</v>
+      </c>
+      <c r="J7" s="2">
+        <f t="shared" si="0"/>
+        <v>0.1368</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B8" s="4">
+        <v>45077</v>
+      </c>
+      <c r="C8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E8" t="s">
+        <v>134</v>
+      </c>
+      <c r="F8" t="s">
+        <v>135</v>
+      </c>
+      <c r="G8" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="1">
+        <v>6100</v>
+      </c>
+      <c r="I8" s="1">
+        <v>544</v>
+      </c>
+      <c r="J8" s="2">
+        <f t="shared" si="0"/>
+        <v>8.9180327868852466E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="4">
+        <v>45077</v>
+      </c>
+      <c r="C9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" t="s">
+        <v>115</v>
+      </c>
+      <c r="E9" t="s">
+        <v>134</v>
+      </c>
+      <c r="F9" t="s">
+        <v>135</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="1">
+        <v>4625</v>
+      </c>
+      <c r="I9" s="1">
+        <v>670</v>
+      </c>
+      <c r="J9" s="2">
+        <f t="shared" si="0"/>
+        <v>0.14486486486486486</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="4">
+        <v>45077</v>
+      </c>
+      <c r="C10" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" t="s">
+        <v>116</v>
+      </c>
+      <c r="E10" t="s">
+        <v>134</v>
+      </c>
+      <c r="F10" t="s">
+        <v>135</v>
+      </c>
+      <c r="G10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" s="1">
+        <v>3800</v>
+      </c>
+      <c r="I10" s="1">
+        <v>2045</v>
+      </c>
+      <c r="J10" s="2">
+        <f t="shared" si="0"/>
+        <v>0.53815789473684206</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="4">
+        <v>45077</v>
+      </c>
+      <c r="C11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" t="s">
+        <v>134</v>
+      </c>
+      <c r="F11" t="s">
+        <v>135</v>
+      </c>
+      <c r="G11" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="1">
+        <v>3600</v>
+      </c>
+      <c r="I11" s="1">
+        <v>1564</v>
+      </c>
+      <c r="J11" s="2">
+        <f t="shared" si="0"/>
+        <v>0.43444444444444447</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="4">
+        <v>45077</v>
+      </c>
+      <c r="C12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" t="s">
+        <v>134</v>
+      </c>
+      <c r="F12" t="s">
+        <v>135</v>
+      </c>
+      <c r="G12" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="1">
+        <v>5100</v>
+      </c>
+      <c r="I12" s="1">
+        <v>1220</v>
+      </c>
+      <c r="J12" s="2">
+        <f t="shared" si="0"/>
+        <v>0.23921568627450981</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B13" s="4">
+        <v>45077</v>
+      </c>
+      <c r="C13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" t="s">
+        <v>117</v>
+      </c>
+      <c r="E13" t="s">
+        <v>134</v>
+      </c>
+      <c r="F13" t="s">
+        <v>135</v>
+      </c>
+      <c r="G13" t="s">
+        <v>50</v>
+      </c>
+      <c r="H13" s="1">
+        <v>4750</v>
+      </c>
+      <c r="I13" s="1">
+        <v>1435</v>
+      </c>
+      <c r="J13" s="2">
+        <f t="shared" si="0"/>
+        <v>0.30210526315789471</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="4">
+        <v>45077</v>
+      </c>
+      <c r="C14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D14" t="s">
+        <v>118</v>
+      </c>
+      <c r="E14" t="s">
+        <v>138</v>
+      </c>
+      <c r="F14" t="s">
+        <v>139</v>
+      </c>
+      <c r="G14" t="s">
+        <v>51</v>
+      </c>
+      <c r="H14" s="1">
+        <v>6000</v>
+      </c>
+      <c r="I14" s="1">
+        <v>998</v>
+      </c>
+      <c r="J14" s="2">
+        <f t="shared" si="0"/>
+        <v>0.16633333333333333</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B15" s="4">
+        <v>45077</v>
+      </c>
+      <c r="C15" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" t="s">
+        <v>119</v>
+      </c>
+      <c r="E15" t="s">
+        <v>140</v>
+      </c>
+      <c r="F15" t="s">
+        <v>141</v>
+      </c>
+      <c r="G15" t="s">
+        <v>50</v>
+      </c>
+      <c r="H15" s="1">
+        <v>4500</v>
+      </c>
+      <c r="I15" s="1">
+        <v>780</v>
+      </c>
+      <c r="J15" s="2">
+        <f t="shared" si="0"/>
+        <v>0.17333333333333334</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B16" s="4">
+        <v>45078</v>
+      </c>
+      <c r="C16" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" t="s">
+        <v>140</v>
+      </c>
+      <c r="F16" t="s">
+        <v>141</v>
+      </c>
+      <c r="G16" t="s">
+        <v>48</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I16" s="1">
+        <v>1044</v>
+      </c>
+      <c r="J16" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B17" s="4">
+        <v>45078</v>
+      </c>
+      <c r="C17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17" t="s">
+        <v>120</v>
+      </c>
+      <c r="E17" t="s">
+        <v>140</v>
+      </c>
+      <c r="F17" t="s">
+        <v>141</v>
+      </c>
+      <c r="G17" t="s">
+        <v>51</v>
+      </c>
+      <c r="H17" s="1">
+        <v>3712.5</v>
+      </c>
+      <c r="I17" s="1">
+        <v>1222</v>
+      </c>
+      <c r="J17" s="2">
+        <f t="shared" si="0"/>
+        <v>0.32915824915824915</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B18" s="4">
+        <v>45078</v>
+      </c>
+      <c r="C18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D18" t="s">
+        <v>121</v>
+      </c>
+      <c r="E18" t="s">
+        <v>140</v>
+      </c>
+      <c r="F18" t="s">
+        <v>141</v>
+      </c>
+      <c r="G18" t="s">
+        <v>51</v>
+      </c>
+      <c r="H18" s="1">
+        <v>4950</v>
+      </c>
+      <c r="I18" s="1">
+        <v>1065</v>
+      </c>
+      <c r="J18" s="2">
+        <f t="shared" si="0"/>
+        <v>0.21515151515151515</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B19" s="4">
+        <v>45078</v>
+      </c>
+      <c r="C19" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" t="s">
+        <v>122</v>
+      </c>
+      <c r="E19" t="s">
+        <v>138</v>
+      </c>
+      <c r="F19" t="s">
+        <v>139</v>
+      </c>
+      <c r="G19" t="s">
+        <v>51</v>
+      </c>
+      <c r="H19" s="1">
+        <v>4750</v>
+      </c>
+      <c r="I19" s="1">
+        <v>810</v>
+      </c>
+      <c r="J19" s="2">
+        <f t="shared" si="0"/>
+        <v>0.17052631578947369</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B20" s="4">
+        <v>45078</v>
+      </c>
+      <c r="C20" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" t="s">
+        <v>123</v>
+      </c>
+      <c r="E20" t="s">
+        <v>138</v>
+      </c>
+      <c r="F20" t="s">
+        <v>139</v>
+      </c>
+      <c r="G20" t="s">
+        <v>51</v>
+      </c>
+      <c r="H20" s="1">
+        <v>7320</v>
+      </c>
+      <c r="I20" s="1">
+        <v>933</v>
+      </c>
+      <c r="J20" s="2">
+        <f t="shared" si="0"/>
+        <v>0.12745901639344262</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B21" s="4">
+        <v>45077</v>
+      </c>
+      <c r="C21" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" t="s">
+        <v>118</v>
+      </c>
+      <c r="E21" t="s">
+        <v>138</v>
+      </c>
+      <c r="F21" t="s">
+        <v>139</v>
+      </c>
+      <c r="G21" t="s">
+        <v>51</v>
+      </c>
+      <c r="H21" s="1">
+        <v>6000</v>
+      </c>
+      <c r="I21" s="1">
+        <v>998</v>
+      </c>
+      <c r="J21" s="2">
+        <f t="shared" si="0"/>
+        <v>0.16633333333333333</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B22" s="4">
+        <v>45077</v>
+      </c>
+      <c r="C22" t="s">
+        <v>92</v>
+      </c>
+      <c r="D22" t="s">
+        <v>119</v>
+      </c>
+      <c r="E22" t="s">
+        <v>140</v>
+      </c>
+      <c r="F22" t="s">
+        <v>141</v>
+      </c>
+      <c r="G22" t="s">
+        <v>50</v>
+      </c>
+      <c r="H22" s="1">
+        <v>4500</v>
+      </c>
+      <c r="I22" s="1">
+        <v>780</v>
+      </c>
+      <c r="J22" s="2">
+        <f t="shared" si="0"/>
+        <v>0.17333333333333334</v>
+      </c>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="4">
+        <v>45078</v>
+      </c>
+      <c r="C23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D23" t="s">
+        <v>124</v>
+      </c>
+      <c r="E23" t="s">
+        <v>140</v>
+      </c>
+      <c r="F23" t="s">
+        <v>141</v>
+      </c>
+      <c r="G23" t="s">
+        <v>51</v>
+      </c>
+      <c r="H23" s="1">
+        <v>5087.5</v>
+      </c>
+      <c r="I23" s="1">
+        <v>655</v>
+      </c>
+      <c r="J23" s="2">
+        <f t="shared" si="0"/>
+        <v>0.12874692874692875</v>
+      </c>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B24" s="4">
+        <v>45078</v>
+      </c>
+      <c r="C24" t="s">
+        <v>99</v>
+      </c>
+      <c r="D24" t="s">
+        <v>125</v>
+      </c>
+      <c r="E24" t="s">
+        <v>140</v>
+      </c>
+      <c r="F24" t="s">
+        <v>141</v>
+      </c>
+      <c r="G24" t="s">
+        <v>51</v>
+      </c>
+      <c r="H24" s="1">
+        <v>4500</v>
+      </c>
+      <c r="I24" s="1">
+        <v>722</v>
+      </c>
+      <c r="J24" s="2">
+        <f t="shared" si="0"/>
+        <v>0.16044444444444445</v>
+      </c>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B25" s="4">
+        <v>45078</v>
+      </c>
+      <c r="C25" t="s">
+        <v>100</v>
+      </c>
+      <c r="D25" t="s">
+        <v>126</v>
+      </c>
+      <c r="E25" t="s">
+        <v>140</v>
+      </c>
+      <c r="F25" t="s">
+        <v>141</v>
+      </c>
+      <c r="G25" t="s">
+        <v>48</v>
+      </c>
+      <c r="H25" s="1">
+        <v>4250</v>
+      </c>
+      <c r="I25" s="1">
+        <v>901</v>
+      </c>
+      <c r="J25" s="2">
+        <f t="shared" si="0"/>
+        <v>0.21199999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B26" s="4">
+        <v>45079</v>
+      </c>
+      <c r="C26" t="s">
+        <v>101</v>
+      </c>
+      <c r="D26" t="s">
+        <v>127</v>
+      </c>
+      <c r="E26" t="s">
+        <v>140</v>
+      </c>
+      <c r="F26" t="s">
+        <v>141</v>
+      </c>
+      <c r="G26" t="s">
+        <v>49</v>
+      </c>
+      <c r="H26" s="1">
+        <v>5250</v>
+      </c>
+      <c r="I26" s="1">
+        <v>1349</v>
+      </c>
+      <c r="J26" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25695238095238093</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B27" s="4">
+        <v>45079</v>
+      </c>
+      <c r="C27" t="s">
+        <v>102</v>
+      </c>
+      <c r="D27" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" t="s">
+        <v>136</v>
+      </c>
+      <c r="F27" t="s">
+        <v>137</v>
+      </c>
+      <c r="G27" t="s">
+        <v>49</v>
+      </c>
+      <c r="H27" s="1">
+        <v>6500</v>
+      </c>
+      <c r="I27" s="1">
+        <v>1288</v>
+      </c>
+      <c r="J27" s="2">
+        <f t="shared" si="0"/>
+        <v>0.19815384615384615</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B28" s="4">
+        <v>45079</v>
+      </c>
+      <c r="C28" t="s">
+        <v>103</v>
+      </c>
+      <c r="D28" t="s">
+        <v>129</v>
+      </c>
+      <c r="E28" t="s">
+        <v>136</v>
+      </c>
+      <c r="F28" t="s">
+        <v>137</v>
+      </c>
+      <c r="G28" t="s">
+        <v>49</v>
+      </c>
+      <c r="H28" s="1">
+        <v>7500</v>
+      </c>
+      <c r="I28" s="1">
+        <v>1664</v>
+      </c>
+      <c r="J28" s="2">
+        <f t="shared" si="0"/>
+        <v>0.22186666666666666</v>
+      </c>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B29" s="4">
+        <v>45079</v>
+      </c>
+      <c r="C29" t="s">
+        <v>104</v>
+      </c>
+      <c r="D29" t="s">
+        <v>130</v>
+      </c>
+      <c r="E29" t="s">
+        <v>136</v>
+      </c>
+      <c r="F29" t="s">
+        <v>137</v>
+      </c>
+      <c r="G29" t="s">
+        <v>51</v>
+      </c>
+      <c r="H29" s="1">
+        <v>5500</v>
+      </c>
+      <c r="I29" s="1">
+        <v>1320</v>
+      </c>
+      <c r="J29" s="2">
+        <f t="shared" si="0"/>
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B30" s="4">
+        <v>45079</v>
+      </c>
+      <c r="C30" t="s">
+        <v>105</v>
+      </c>
+      <c r="D30" t="s">
+        <v>131</v>
+      </c>
+      <c r="E30" t="s">
+        <v>136</v>
+      </c>
+      <c r="F30" t="s">
+        <v>137</v>
+      </c>
+      <c r="G30" t="s">
+        <v>51</v>
+      </c>
+      <c r="H30" s="1">
+        <v>4625</v>
+      </c>
+      <c r="I30" s="1">
+        <v>1001</v>
+      </c>
+      <c r="J30" s="2">
+        <f t="shared" si="0"/>
+        <v>0.21643243243243243</v>
+      </c>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B31" s="4">
+        <v>45079</v>
+      </c>
+      <c r="C31" t="s">
+        <v>106</v>
+      </c>
+      <c r="D31" t="s">
+        <v>132</v>
+      </c>
+      <c r="E31" t="s">
+        <v>136</v>
+      </c>
+      <c r="F31" t="s">
+        <v>137</v>
+      </c>
+      <c r="G31" t="s">
+        <v>51</v>
+      </c>
+      <c r="H31" s="1">
+        <v>4500</v>
+      </c>
+      <c r="I31" s="1">
+        <v>960</v>
+      </c>
+      <c r="J31" s="2">
+        <f t="shared" si="0"/>
+        <v>0.21333333333333335</v>
+      </c>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B32" s="4">
+        <v>45079</v>
+      </c>
+      <c r="C32" t="s">
+        <v>107</v>
+      </c>
+      <c r="D32" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32" t="s">
+        <v>136</v>
+      </c>
+      <c r="F32" t="s">
+        <v>137</v>
+      </c>
+      <c r="G32" t="s">
+        <v>48</v>
+      </c>
+      <c r="H32" s="1">
+        <v>5400</v>
+      </c>
+      <c r="I32" s="1">
+        <v>540</v>
+      </c>
+      <c r="J32" s="2">
+        <f t="shared" si="0"/>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B33" s="4">
+        <v>45076</v>
+      </c>
+      <c r="C33" t="s">
+        <v>84</v>
+      </c>
+      <c r="D33" t="s">
+        <v>113</v>
+      </c>
+      <c r="E33" t="s">
+        <v>138</v>
+      </c>
+      <c r="F33" t="s">
+        <v>139</v>
+      </c>
+      <c r="G33" t="s">
+        <v>50</v>
+      </c>
+      <c r="H33" s="1">
+        <v>5000</v>
+      </c>
+      <c r="I33" s="1">
+        <v>684</v>
+      </c>
+      <c r="J33" s="2">
+        <f t="shared" si="0"/>
+        <v>0.1368</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>142</v>
+      </c>
+      <c r="C34" t="s">
+        <v>108</v>
+      </c>
+      <c r="D34" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" t="s">
+        <v>142</v>
+      </c>
+      <c r="F34" t="s">
+        <v>142</v>
+      </c>
+      <c r="G34" t="s">
+        <v>142</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I34" t="s">
+        <v>142</v>
+      </c>
+      <c r="J34" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>142</v>
+      </c>
+      <c r="C35" t="s">
+        <v>108</v>
+      </c>
+      <c r="D35" t="s">
+        <v>108</v>
+      </c>
+      <c r="E35" t="s">
+        <v>142</v>
+      </c>
+      <c r="F35" t="s">
+        <v>142</v>
+      </c>
+      <c r="G35" t="s">
+        <v>142</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I35" t="s">
+        <v>142</v>
+      </c>
+      <c r="J35" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H36" s="1"/>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H37" s="1"/>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H38" s="1"/>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H39" s="1"/>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H40" s="1"/>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H42" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>